<commit_message>
fix(ai): fix future covariates missing date
</commit_message>
<xml_diff>
--- a/reports/tft_prediction_results.xlsx
+++ b/reports/tft_prediction_results.xlsx
@@ -511,19 +511,19 @@
         <v>23.4</v>
       </c>
       <c r="G2" t="n">
-        <v>64.65365600585938</v>
+        <v>59.74925231933594</v>
       </c>
       <c r="H2" t="n">
-        <v>64.80541229248047</v>
+        <v>55.073486328125</v>
       </c>
       <c r="I2" t="n">
-        <v>2530.16552734375</v>
+        <v>2467.5283203125</v>
       </c>
       <c r="J2" t="n">
-        <v>59.79232406616211</v>
+        <v>53.70585632324219</v>
       </c>
       <c r="K2" t="n">
-        <v>16.90903854370117</v>
+        <v>18.07442855834961</v>
       </c>
     </row>
     <row r="3">
@@ -546,19 +546,19 @@
         <v>23.5</v>
       </c>
       <c r="G3" t="n">
-        <v>56.2020263671875</v>
+        <v>52.70097351074219</v>
       </c>
       <c r="H3" t="n">
-        <v>61.30005264282227</v>
+        <v>51.13645172119141</v>
       </c>
       <c r="I3" t="n">
-        <v>2099.528076171875</v>
+        <v>1333.216430664062</v>
       </c>
       <c r="J3" t="n">
-        <v>64.9388427734375</v>
+        <v>55.67532730102539</v>
       </c>
       <c r="K3" t="n">
-        <v>14.11795520782471</v>
+        <v>13.2206335067749</v>
       </c>
     </row>
     <row r="4">
@@ -581,19 +581,19 @@
         <v>22.9</v>
       </c>
       <c r="G4" t="n">
-        <v>61.89712524414062</v>
+        <v>67.44716644287109</v>
       </c>
       <c r="H4" t="n">
-        <v>64.27066040039062</v>
+        <v>64.02257537841797</v>
       </c>
       <c r="I4" t="n">
-        <v>2642.767333984375</v>
+        <v>1779.318237304688</v>
       </c>
       <c r="J4" t="n">
-        <v>51.39938354492188</v>
+        <v>49.13541030883789</v>
       </c>
       <c r="K4" t="n">
-        <v>18.99428749084473</v>
+        <v>18.03343772888184</v>
       </c>
     </row>
     <row r="5">
@@ -616,19 +616,19 @@
         <v>22</v>
       </c>
       <c r="G5" t="n">
-        <v>62.54704284667969</v>
+        <v>74.05523681640625</v>
       </c>
       <c r="H5" t="n">
-        <v>61.77443313598633</v>
+        <v>71.88275909423828</v>
       </c>
       <c r="I5" t="n">
-        <v>1878.63916015625</v>
+        <v>1189.161987304688</v>
       </c>
       <c r="J5" t="n">
-        <v>55.03580474853516</v>
+        <v>48.65460205078125</v>
       </c>
       <c r="K5" t="n">
-        <v>19.06656265258789</v>
+        <v>16.65051078796387</v>
       </c>
     </row>
     <row r="6">
@@ -651,19 +651,19 @@
         <v>21</v>
       </c>
       <c r="G6" t="n">
-        <v>61.09850311279297</v>
+        <v>74.58026123046875</v>
       </c>
       <c r="H6" t="n">
-        <v>62.31778717041016</v>
+        <v>76.25457000732422</v>
       </c>
       <c r="I6" t="n">
-        <v>1478.9853515625</v>
+        <v>934.002197265625</v>
       </c>
       <c r="J6" t="n">
-        <v>46.34407043457031</v>
+        <v>42.94955062866211</v>
       </c>
       <c r="K6" t="n">
-        <v>13.53823661804199</v>
+        <v>11.42043399810791</v>
       </c>
     </row>
     <row r="7">
@@ -686,19 +686,19 @@
         <v>20</v>
       </c>
       <c r="G7" t="n">
-        <v>49.93083190917969</v>
+        <v>61.35310745239258</v>
       </c>
       <c r="H7" t="n">
-        <v>87.70808410644531</v>
+        <v>110.2657165527344</v>
       </c>
       <c r="I7" t="n">
-        <v>1105.797241210938</v>
+        <v>751.6087646484375</v>
       </c>
       <c r="J7" t="n">
-        <v>48.74736785888672</v>
+        <v>45.63566207885742</v>
       </c>
       <c r="K7" t="n">
-        <v>22.34971618652344</v>
+        <v>19.59607887268066</v>
       </c>
     </row>
     <row r="8">
@@ -721,19 +721,19 @@
         <v>19</v>
       </c>
       <c r="G8" t="n">
-        <v>59.8266487121582</v>
+        <v>72.98283386230469</v>
       </c>
       <c r="H8" t="n">
-        <v>68.16487884521484</v>
+        <v>82.51547241210938</v>
       </c>
       <c r="I8" t="n">
-        <v>1348.689086914062</v>
+        <v>991.6757202148438</v>
       </c>
       <c r="J8" t="n">
-        <v>46.32328033447266</v>
+        <v>43.29195785522461</v>
       </c>
       <c r="K8" t="n">
-        <v>27.9713249206543</v>
+        <v>28.54887962341309</v>
       </c>
     </row>
     <row r="9">
@@ -756,19 +756,19 @@
         <v>18.6</v>
       </c>
       <c r="G9" t="n">
-        <v>57.84267044067383</v>
+        <v>70.95880889892578</v>
       </c>
       <c r="H9" t="n">
-        <v>80.1510009765625</v>
+        <v>98.31162261962891</v>
       </c>
       <c r="I9" t="n">
-        <v>1128.9228515625</v>
+        <v>904.0664672851562</v>
       </c>
       <c r="J9" t="n">
-        <v>28.2955379486084</v>
+        <v>24.75147819519043</v>
       </c>
       <c r="K9" t="n">
-        <v>17.36457252502441</v>
+        <v>17.07504653930664</v>
       </c>
     </row>
     <row r="10">
@@ -791,19 +791,19 @@
         <v>18.9</v>
       </c>
       <c r="G10" t="n">
-        <v>45.90960311889648</v>
+        <v>56.80191421508789</v>
       </c>
       <c r="H10" t="n">
-        <v>58.45135879516602</v>
+        <v>70.90772247314453</v>
       </c>
       <c r="I10" t="n">
-        <v>1035.330688476562</v>
+        <v>1011.109375</v>
       </c>
       <c r="J10" t="n">
-        <v>35.29219436645508</v>
+        <v>34.41070556640625</v>
       </c>
       <c r="K10" t="n">
-        <v>16.41268730163574</v>
+        <v>18.12965965270996</v>
       </c>
     </row>
     <row r="11">
@@ -826,19 +826,19 @@
         <v>19.8</v>
       </c>
       <c r="G11" t="n">
-        <v>57.11300277709961</v>
+        <v>68.27223205566406</v>
       </c>
       <c r="H11" t="n">
-        <v>76.24634552001953</v>
+        <v>88.88423919677734</v>
       </c>
       <c r="I11" t="n">
-        <v>1160.932373046875</v>
+        <v>1188.715698242188</v>
       </c>
       <c r="J11" t="n">
-        <v>33.13983535766602</v>
+        <v>34.08225631713867</v>
       </c>
       <c r="K11" t="n">
-        <v>21.48879623413086</v>
+        <v>23.74041366577148</v>
       </c>
     </row>
     <row r="12">
@@ -861,19 +861,19 @@
         <v>24.2</v>
       </c>
       <c r="G12" t="n">
-        <v>64.64549255371094</v>
+        <v>76.31001281738281</v>
       </c>
       <c r="H12" t="n">
-        <v>51.30139923095703</v>
+        <v>51.40607452392578</v>
       </c>
       <c r="I12" t="n">
-        <v>1292.855346679688</v>
+        <v>1452.523071289062</v>
       </c>
       <c r="J12" t="n">
-        <v>46.31076812744141</v>
+        <v>55.63755798339844</v>
       </c>
       <c r="K12" t="n">
-        <v>21.73600196838379</v>
+        <v>29.07956886291504</v>
       </c>
     </row>
     <row r="13">
@@ -896,19 +896,19 @@
         <v>30.8</v>
       </c>
       <c r="G13" t="n">
-        <v>40.79114151000977</v>
+        <v>47.10625839233398</v>
       </c>
       <c r="H13" t="n">
-        <v>46.78893280029297</v>
+        <v>50.49948883056641</v>
       </c>
       <c r="I13" t="n">
-        <v>1361.312255859375</v>
+        <v>1614.970458984375</v>
       </c>
       <c r="J13" t="n">
-        <v>30.11051940917969</v>
+        <v>37.42718887329102</v>
       </c>
       <c r="K13" t="n">
-        <v>14.99010372161865</v>
+        <v>21.7042236328125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>